<commit_message>
BUG008 to BUG010 Added
</commit_message>
<xml_diff>
--- a/Bug Reports/BugReport.xlsx
+++ b/Bug Reports/BugReport.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="63">
   <si>
     <t>Bug ID</t>
   </si>
@@ -201,6 +201,85 @@
   <si>
     <t>No validation message was displayed when
 the user attended post with empty content.</t>
+  </si>
+  <si>
+    <t>BUG008</t>
+  </si>
+  <si>
+    <t>BUG009</t>
+  </si>
+  <si>
+    <t>BUG010</t>
+  </si>
+  <si>
+    <t>Account is not locked after multiple failed
+login attempts</t>
+  </si>
+  <si>
+    <t>1. Navigate to the login page.
+2. Enter a valid username.
+3. Enter an incorrect password
+multiple times (e.g., 10-15 
+consective attempts).
+4. Observe the system behavior.</t>
+  </si>
+  <si>
+    <t>The account should be temporarily locked
+or restricted after multiple failed login
+attempts, and an appropriate lockout
+message should be displayed.</t>
+  </si>
+  <si>
+    <t>The system continuosly displayed the 
+"Invalid credentials" message and does not
+lock or restrict the account after multiple
+failed attempts.</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>User can access Dashboard directly after
+logout</t>
+  </si>
+  <si>
+    <t>1. Login to the application.
+2. Logout from the application.
+3. Directly access a protected 
+URL (e.g., Dashboard URL).</t>
+  </si>
+  <si>
+    <t>User should be redirected to the login page
+when attempting to access a protected
+URL after logout.</t>
+  </si>
+  <si>
+    <t>User was redirected to the Dashboard and 
+cpuld access the appliaction even after
+logout.</t>
+  </si>
+  <si>
+    <t>Protected pages are accessible using browser
+Back button after logout.</t>
+  </si>
+  <si>
+    <t>1. Login to the application.
+2. Logout from the application.
+3. Click the browser Back 
+button.
+4. Observe whether protected
+pages are accessible.</t>
+  </si>
+  <si>
+    <t>Protected pages should not be accessible
+after logout. The user should be redirected
+to the Login page or shown access denined
+message.</t>
+  </si>
+  <si>
+    <t>Protected page remained accessible after
+logout when the browser Back button was
+used.</t>
   </si>
 </sst>
 </file>
@@ -533,7 +612,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="38.7265625" bestFit="1" customWidth="1"/>
@@ -753,6 +832,84 @@
         <v>13</v>
       </c>
     </row>
+    <row r="9" spans="1:8" ht="116" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>